<commit_message>
feat: update sample data in purchases CSV and enhance demo script instructions
</commit_message>
<xml_diff>
--- a/demo/samples/bearings/01-sales-register.xlsx
+++ b/demo/samples/bearings/01-sales-register.xlsx
@@ -500,7 +500,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -536,7 +536,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>09-03-2026</t>
+          <t>14-03-2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -612,7 +612,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -648,7 +648,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -688,7 +688,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -728,7 +728,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -764,7 +764,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14-04-2026</t>
+          <t>19-04-2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -804,7 +804,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>30-08-2026</t>
+          <t>04-09-2026</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -840,7 +840,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>01-04-2026</t>
+          <t>06-04-2026</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -876,7 +876,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>20-08-2026</t>
+          <t>25-08-2026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -916,7 +916,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>14-07-2026</t>
+          <t>19-07-2026</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -952,7 +952,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -988,7 +988,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10-07-2026</t>
+          <t>15-07-2026</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1028,7 +1028,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>29-03-2026</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1068,7 +1068,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1104,7 +1104,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>10-03-2026</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1140,7 +1140,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1180,7 +1180,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1220,7 +1220,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>25-04-2026</t>
+          <t>30-04-2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1260,7 +1260,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>07-09-2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1300,7 +1300,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>02-05-2026</t>
+          <t>07-05-2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1336,7 +1336,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>22-07-2026</t>
+          <t>27-07-2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1376,7 +1376,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>24-04-2026</t>
+          <t>29-04-2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1412,7 +1412,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1452,7 +1452,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>03-08-2026</t>
+          <t>08-08-2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1488,7 +1488,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1524,7 +1524,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1560,7 +1560,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1596,7 +1596,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>27-07-2026</t>
+          <t>01-08-2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1632,7 +1632,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1668,7 +1668,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1704,7 +1704,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1744,7 +1744,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1784,7 +1784,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1820,7 +1820,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1860,7 +1860,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1900,7 +1900,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>13-03-2026</t>
+          <t>18-03-2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1940,7 +1940,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>13-07-2026</t>
+          <t>18-07-2026</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1980,7 +1980,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2020,7 +2020,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2060,7 +2060,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2096,7 +2096,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>18-07-2026</t>
+          <t>23-07-2026</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2132,7 +2132,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2172,7 +2172,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2212,7 +2212,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2248,7 +2248,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>04-07-2026</t>
+          <t>09-07-2026</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2288,7 +2288,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2328,7 +2328,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08-03-2026</t>
+          <t>13-03-2026</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2368,7 +2368,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>12-09-2026</t>
+          <t>17-09-2026</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2408,7 +2408,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08-04-2026</t>
+          <t>13-04-2026</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2448,7 +2448,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>07-09-2026</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2484,7 +2484,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2524,7 +2524,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>25-03-2026</t>
+          <t>30-03-2026</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2564,7 +2564,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2600,7 +2600,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2636,7 +2636,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2676,7 +2676,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>09-06-2026</t>
+          <t>14-06-2026</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2716,7 +2716,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2756,7 +2756,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>05-07-2026</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2792,7 +2792,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2828,7 +2828,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>28-03-2026</t>
+          <t>02-04-2026</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2864,7 +2864,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>13-09-2026</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2904,7 +2904,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>09-06-2026</t>
+          <t>14-06-2026</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2940,7 +2940,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2980,7 +2980,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3020,7 +3020,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>30-05-2026</t>
+          <t>04-06-2026</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3056,7 +3056,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3092,7 +3092,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3128,7 +3128,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>21-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3168,7 +3168,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>21-05-2026</t>
+          <t>26-05-2026</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3208,7 +3208,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3244,7 +3244,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>19-05-2026</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3284,7 +3284,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3320,7 +3320,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>11-06-2026</t>
+          <t>16-06-2026</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3360,7 +3360,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>29-03-2026</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3400,7 +3400,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3436,7 +3436,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>19-07-2026</t>
+          <t>24-07-2026</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3472,7 +3472,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3512,7 +3512,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>12-04-2026</t>
+          <t>17-04-2026</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3552,7 +3552,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -3592,7 +3592,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3632,7 +3632,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -3668,7 +3668,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -3704,7 +3704,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -3744,7 +3744,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>03-04-2026</t>
+          <t>08-04-2026</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -3780,7 +3780,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -3816,7 +3816,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>31-05-2026</t>
+          <t>05-06-2026</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3852,7 +3852,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>20-04-2026</t>
+          <t>25-04-2026</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -3888,7 +3888,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -3928,7 +3928,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>16-08-2026</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3968,7 +3968,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>13-03-2026</t>
+          <t>18-03-2026</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4008,7 +4008,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4048,7 +4048,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4084,7 +4084,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4124,7 +4124,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>14-09-2026</t>
+          <t>19-09-2026</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4164,7 +4164,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>18-08-2026</t>
+          <t>23-08-2026</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -4204,7 +4204,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
+          <t>13-06-2026</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4240,7 +4240,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>07-05-2026</t>
+          <t>12-05-2026</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -4280,7 +4280,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4316,7 +4316,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -4356,7 +4356,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>22-03-2026</t>
+          <t>27-03-2026</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -4392,7 +4392,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>24-07-2026</t>
+          <t>29-07-2026</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -4428,7 +4428,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -4464,7 +4464,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -4500,7 +4500,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>02-05-2026</t>
+          <t>07-05-2026</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -4540,7 +4540,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>15-04-2026</t>
+          <t>20-04-2026</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -4576,7 +4576,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>25-03-2026</t>
+          <t>30-03-2026</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -4616,7 +4616,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -4656,7 +4656,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>11-07-2026</t>
+          <t>16-07-2026</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -4692,7 +4692,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>06-07-2026</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -4732,7 +4732,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -4772,7 +4772,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -4808,7 +4808,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -4844,7 +4844,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>22-08-2026</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -4884,7 +4884,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>31-03-2026</t>
+          <t>05-04-2026</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -4920,7 +4920,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -4956,7 +4956,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>17-04-2026</t>
+          <t>22-04-2026</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -4996,7 +4996,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -5036,7 +5036,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -5072,7 +5072,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -5108,7 +5108,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -5144,7 +5144,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>25-05-2026</t>
+          <t>30-05-2026</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -5184,7 +5184,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>22-08-2026</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -5220,7 +5220,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -5260,7 +5260,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -5296,7 +5296,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>05-07-2026</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -5332,7 +5332,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -5368,7 +5368,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -5404,7 +5404,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>24-05-2026</t>
+          <t>29-05-2026</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -5444,7 +5444,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -5484,7 +5484,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13-05-2026</t>
+          <t>18-05-2026</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -5524,7 +5524,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>18-03-2026</t>
+          <t>23-03-2026</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -5564,7 +5564,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>27-08-2026</t>
+          <t>01-09-2026</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -5604,7 +5604,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -5644,7 +5644,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>26-08-2026</t>
+          <t>31-08-2026</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -5684,7 +5684,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -5720,7 +5720,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -5756,7 +5756,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -5796,7 +5796,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -5832,7 +5832,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -5872,7 +5872,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -5908,7 +5908,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -5944,7 +5944,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -5980,7 +5980,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -6016,7 +6016,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -6052,7 +6052,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -6092,7 +6092,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>13-07-2026</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -6132,7 +6132,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>08-07-2026</t>
+          <t>13-07-2026</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -6172,7 +6172,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -6212,7 +6212,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>23-08-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -6270,7 +6270,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>19-05-2026</t>
+          <t>24-05-2026</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -6310,7 +6310,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -6350,7 +6350,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>10-03-2026</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -6386,7 +6386,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>25-05-2026</t>
+          <t>30-05-2026</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -6422,7 +6422,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -6462,7 +6462,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -6498,7 +6498,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -6538,7 +6538,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -6578,7 +6578,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -6614,7 +6614,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -6650,7 +6650,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -6690,7 +6690,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>12-09-2026</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -6730,7 +6730,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -6770,7 +6770,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>23-05-2026</t>
+          <t>28-05-2026</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -6810,7 +6810,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -6846,7 +6846,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>22-08-2026</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -6882,7 +6882,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -6918,7 +6918,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -6954,7 +6954,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>21-05-2026</t>
+          <t>26-05-2026</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -6990,7 +6990,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>27-04-2026</t>
+          <t>02-05-2026</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -7026,7 +7026,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>17-04-2026</t>
+          <t>22-04-2026</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -7066,7 +7066,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>21-04-2026</t>
+          <t>26-04-2026</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -7102,7 +7102,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -7142,7 +7142,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -7182,7 +7182,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>01-08-2026</t>
+          <t>06-08-2026</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -7222,7 +7222,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -7258,7 +7258,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -7298,7 +7298,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -7338,7 +7338,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>15-08-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -7374,7 +7374,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>07-04-2026</t>
+          <t>12-04-2026</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -7414,7 +7414,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -7454,7 +7454,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>14-05-2026</t>
+          <t>19-05-2026</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -7490,7 +7490,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -7530,7 +7530,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>07-03-2026</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -7570,7 +7570,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -7606,7 +7606,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>21-06-2026</t>
+          <t>26-06-2026</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -7642,7 +7642,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>05-08-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -7682,7 +7682,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>08-05-2026</t>
+          <t>13-05-2026</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -7718,7 +7718,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -7754,7 +7754,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>21-04-2026</t>
+          <t>26-04-2026</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -7790,7 +7790,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>06-07-2026</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -7826,7 +7826,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -7862,7 +7862,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>05-07-2026</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -7898,7 +7898,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>13-08-2026</t>
+          <t>18-08-2026</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -7934,7 +7934,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -7970,7 +7970,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -8010,7 +8010,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>02-07-2026</t>
+          <t>07-07-2026</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -8046,7 +8046,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -8082,7 +8082,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -8118,7 +8118,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -8154,7 +8154,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>23-07-2026</t>
+          <t>28-07-2026</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -8190,7 +8190,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>12-09-2026</t>
+          <t>17-09-2026</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -8230,7 +8230,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>05-07-2026</t>
+          <t>10-07-2026</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -8266,7 +8266,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>08-03-2026</t>
+          <t>13-03-2026</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -8302,7 +8302,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -8342,7 +8342,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -8382,7 +8382,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -8418,7 +8418,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>11-05-2026</t>
+          <t>16-05-2026</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -8458,7 +8458,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -8498,7 +8498,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>15-05-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -8538,7 +8538,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -8578,7 +8578,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -8614,7 +8614,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>23-05-2026</t>
+          <t>28-05-2026</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -8654,7 +8654,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>24-05-2026</t>
+          <t>29-05-2026</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -8690,7 +8690,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -8730,7 +8730,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>15-06-2026</t>
+          <t>20-06-2026</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -8766,7 +8766,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -8802,7 +8802,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>06-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -8842,7 +8842,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>13-05-2026</t>
+          <t>18-05-2026</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -8878,7 +8878,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>24-03-2026</t>
+          <t>29-03-2026</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -8914,7 +8914,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>04-06-2026</t>
+          <t>09-06-2026</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -8950,7 +8950,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -8990,7 +8990,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>28-06-2026</t>
+          <t>03-07-2026</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -9026,7 +9026,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -9066,7 +9066,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -9106,7 +9106,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>13-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -9142,7 +9142,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>06-04-2026</t>
+          <t>11-04-2026</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -9178,7 +9178,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>10-05-2026</t>
+          <t>15-05-2026</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -9214,7 +9214,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -9250,7 +9250,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -9290,7 +9290,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -9326,7 +9326,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -9362,7 +9362,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -9402,7 +9402,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -9442,7 +9442,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>16-08-2026</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -9478,7 +9478,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -9514,7 +9514,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>07-09-2026</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -9550,7 +9550,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -9590,7 +9590,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -9626,7 +9626,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>08-04-2026</t>
+          <t>13-04-2026</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -9666,7 +9666,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>27-03-2026</t>
+          <t>01-04-2026</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -9702,7 +9702,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>20-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -9738,7 +9738,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -9778,7 +9778,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>13-09-2026</t>
+          <t>18-09-2026</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -9818,7 +9818,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -9858,7 +9858,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -9898,7 +9898,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>06-04-2026</t>
+          <t>11-04-2026</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -9934,7 +9934,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -9974,7 +9974,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>05-07-2026</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -10010,7 +10010,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -10046,7 +10046,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>25-07-2026</t>
+          <t>30-07-2026</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -10082,7 +10082,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -10118,7 +10118,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>31-08-2026</t>
+          <t>05-09-2026</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -10154,7 +10154,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>14-09-2026</t>
+          <t>19-09-2026</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -10190,7 +10190,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -10230,7 +10230,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -10270,7 +10270,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>08-04-2026</t>
+          <t>13-04-2026</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -10310,7 +10310,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>23-06-2026</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -10350,7 +10350,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>05-03-2026</t>
+          <t>10-03-2026</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">

</xml_diff>